<commit_message>
list properties should not have filters
</commit_message>
<xml_diff>
--- a/src/ExcelsiorClosedXml.Tests/ComplexTypeWithCustomEnumerableRender.Null.verified.xlsx
+++ b/src/ExcelsiorClosedXml.Tests/ComplexTypeWithCustomEnumerableRender.Null.verified.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="DeterministicId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$B$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$2</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -416,7 +416,7 @@
       <c r="B2" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B2"/>
+  <autoFilter ref="A1:A2"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>

</xml_diff>

<commit_message>
List properties should not have filters (#142)
* list properties should not have filters

* .
</commit_message>
<xml_diff>
--- a/src/ExcelsiorClosedXml.Tests/ComplexTypeWithCustomEnumerableRender.Null.verified.xlsx
+++ b/src/ExcelsiorClosedXml.Tests/ComplexTypeWithCustomEnumerableRender.Null.verified.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="DeterministicId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$B$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$2</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -416,7 +416,7 @@
       <c r="B2" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B2"/>
+  <autoFilter ref="A1:A2"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>

</xml_diff>